<commit_message>
Reorder expiry columns and drop 入力者 from the Excel template
Per feedback: ingredient sheets now run 期限日 / 期限区分 / 期限量 /
期限切れ量 / 期限切れ日 / チェック / 備考, and the 入力者 column and
its 設定 sheet are removed (SharePoint version history already tracks
editors). Formulas, dropdowns, conditional formatting, and summary
counters follow the new layout; re-verified by evaluation.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgvGiotwKBR4F3r5Tdot14
</commit_message>
<xml_diff>
--- a/excel/棚卸しシート_共同編集版.xlsx
+++ b/excel/棚卸しシート_共同編集版.xlsx
@@ -11,7 +11,6 @@
     <sheet name="原料豆" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="副原料" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="フィルター" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="設定" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -581,11 +580,11 @@
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(原料豆!$K$4:$K$41,"1回目完了")</f>
+        <f>COUNTIF(原料豆!$J$4:$J$41,"1回目完了")</f>
         <v/>
       </c>
       <c r="F5" s="6">
-        <f>COUNTIF(原料豆!$K$4:$K$41,"ダブルチェック完了")</f>
+        <f>COUNTIF(原料豆!$J$4:$J$41,"ダブルチェック完了")</f>
         <v/>
       </c>
     </row>
@@ -607,11 +606,11 @@
         <v/>
       </c>
       <c r="E6" s="6">
-        <f>COUNTIF(副原料!$K$4:$K$90,"1回目完了")</f>
+        <f>COUNTIF(副原料!$J$4:$J$90,"1回目完了")</f>
         <v/>
       </c>
       <c r="F6" s="6">
-        <f>COUNTIF(副原料!$K$4:$K$90,"ダブルチェック完了")</f>
+        <f>COUNTIF(副原料!$J$4:$J$90,"ダブルチェック完了")</f>
         <v/>
       </c>
     </row>
@@ -633,11 +632,11 @@
         <v/>
       </c>
       <c r="E7" s="6">
-        <f>COUNTIF(フィルター!$G$4:$G$17,"1回目完了")</f>
+        <f>COUNTIF(フィルター!$F$4:$F$17,"1回目完了")</f>
         <v/>
       </c>
       <c r="F7" s="6">
-        <f>COUNTIF(フィルター!$G$4:$G$17,"ダブルチェック完了")</f>
+        <f>COUNTIF(フィルター!$F$4:$F$17,"ダブルチェック完了")</f>
         <v/>
       </c>
     </row>
@@ -699,7 +698,7 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>4. 入力したら「入力者」を選び、確認が済んだら「チェック」を選ぶ</t>
+          <t>4. 確認が済んだら「チェック」を選ぶ（誰が編集したかはSharePointの版履歴で確認できる）</t>
         </is>
       </c>
     </row>
@@ -735,21 +734,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -793,40 +791,35 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
+          <t>期限日</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>期限区分(自動)</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>期限量</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
           <t>期限切れ量</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>期限切れ日</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>期限日</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>期限区分(自動)</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>期限量</t>
-        </is>
-      </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>入力者</t>
+          <t>チェック</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>チェック</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
@@ -849,17 +842,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="6">
-        <f>IF($G4="","",IF(EDATE(サマリ!$B$2,1)&gt;$G4,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G4,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G4,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I4" s="6" t="n"/>
+      <c r="E4" s="10" t="n"/>
+      <c r="F4" s="6">
+        <f>IF($E4="","",IF(EDATE(サマリ!$B$2,1)&gt;$E4,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E4,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E4,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="10" t="n"/>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -878,17 +870,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="6">
-        <f>IF($G5="","",IF(EDATE(サマリ!$B$2,1)&gt;$G5,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G5,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G5,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I5" s="6" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="6">
+        <f>IF($E5="","",IF(EDATE(サマリ!$B$2,1)&gt;$E5,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E5,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E5,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="10" t="n"/>
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="6" t="n"/>
-      <c r="L5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -907,17 +898,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="6">
-        <f>IF($G6="","",IF(EDATE(サマリ!$B$2,1)&gt;$G6,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G6,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G6,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I6" s="6" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="6">
+        <f>IF($E6="","",IF(EDATE(サマリ!$B$2,1)&gt;$E6,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E6,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E6,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="10" t="n"/>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -936,17 +926,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="6">
-        <f>IF($G7="","",IF(EDATE(サマリ!$B$2,1)&gt;$G7,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G7,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G7,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I7" s="6" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="6">
+        <f>IF($E7="","",IF(EDATE(サマリ!$B$2,1)&gt;$E7,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E7,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E7,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="10" t="n"/>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
-      <c r="L7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -965,17 +954,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="6">
-        <f>IF($G8="","",IF(EDATE(サマリ!$B$2,1)&gt;$G8,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G8,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G8,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I8" s="6" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="6">
+        <f>IF($E8="","",IF(EDATE(サマリ!$B$2,1)&gt;$E8,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E8,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E8,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="10" t="n"/>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
-      <c r="L8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -994,17 +982,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="6">
-        <f>IF($G9="","",IF(EDATE(サマリ!$B$2,1)&gt;$G9,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G9,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G9,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I9" s="6" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="6">
+        <f>IF($E9="","",IF(EDATE(サマリ!$B$2,1)&gt;$E9,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E9,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E9,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="10" t="n"/>
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="6" t="n"/>
-      <c r="L9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -1023,17 +1010,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="6">
-        <f>IF($G10="","",IF(EDATE(サマリ!$B$2,1)&gt;$G10,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G10,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G10,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I10" s="6" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="6">
+        <f>IF($E10="","",IF(EDATE(サマリ!$B$2,1)&gt;$E10,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E10,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E10,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="10" t="n"/>
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
-      <c r="L10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1052,17 +1038,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
-      <c r="H11" s="6">
-        <f>IF($G11="","",IF(EDATE(サマリ!$B$2,1)&gt;$G11,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G11,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G11,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I11" s="6" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="6">
+        <f>IF($E11="","",IF(EDATE(サマリ!$B$2,1)&gt;$E11,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E11,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E11,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="10" t="n"/>
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
-      <c r="L11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -1081,17 +1066,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="6">
-        <f>IF($G12="","",IF(EDATE(サマリ!$B$2,1)&gt;$G12,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G12,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G12,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I12" s="6" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="6">
+        <f>IF($E12="","",IF(EDATE(サマリ!$B$2,1)&gt;$E12,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E12,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E12,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="10" t="n"/>
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
-      <c r="L12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -1110,17 +1094,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
-      <c r="H13" s="6">
-        <f>IF($G13="","",IF(EDATE(サマリ!$B$2,1)&gt;$G13,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G13,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G13,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I13" s="6" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="6">
+        <f>IF($E13="","",IF(EDATE(サマリ!$B$2,1)&gt;$E13,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E13,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E13,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="10" t="n"/>
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
-      <c r="L13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -1139,17 +1122,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="6">
-        <f>IF($G14="","",IF(EDATE(サマリ!$B$2,1)&gt;$G14,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G14,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G14,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I14" s="6" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="6">
+        <f>IF($E14="","",IF(EDATE(サマリ!$B$2,1)&gt;$E14,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E14,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E14,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="10" t="n"/>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
-      <c r="L14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -1168,17 +1150,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="6">
-        <f>IF($G15="","",IF(EDATE(サマリ!$B$2,1)&gt;$G15,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G15,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G15,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I15" s="6" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="6">
+        <f>IF($E15="","",IF(EDATE(サマリ!$B$2,1)&gt;$E15,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E15,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E15,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="10" t="n"/>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
-      <c r="L15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1197,17 +1178,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="6">
-        <f>IF($G16="","",IF(EDATE(サマリ!$B$2,1)&gt;$G16,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G16,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G16,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I16" s="6" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="6">
+        <f>IF($E16="","",IF(EDATE(サマリ!$B$2,1)&gt;$E16,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E16,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E16,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="10" t="n"/>
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
-      <c r="L16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -1226,17 +1206,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
-      <c r="H17" s="6">
-        <f>IF($G17="","",IF(EDATE(サマリ!$B$2,1)&gt;$G17,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G17,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G17,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I17" s="6" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="6">
+        <f>IF($E17="","",IF(EDATE(サマリ!$B$2,1)&gt;$E17,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E17,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E17,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="10" t="n"/>
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
-      <c r="L17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1255,17 +1234,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="6">
-        <f>IF($G18="","",IF(EDATE(サマリ!$B$2,1)&gt;$G18,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G18,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G18,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I18" s="6" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="6">
+        <f>IF($E18="","",IF(EDATE(サマリ!$B$2,1)&gt;$E18,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E18,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E18,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="10" t="n"/>
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
-      <c r="L18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -1284,17 +1262,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="6">
-        <f>IF($G19="","",IF(EDATE(サマリ!$B$2,1)&gt;$G19,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G19,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G19,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I19" s="6" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="6">
+        <f>IF($E19="","",IF(EDATE(サマリ!$B$2,1)&gt;$E19,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E19,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E19,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="10" t="n"/>
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
-      <c r="L19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1313,17 +1290,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="6">
-        <f>IF($G20="","",IF(EDATE(サマリ!$B$2,1)&gt;$G20,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G20,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G20,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I20" s="6" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="6">
+        <f>IF($E20="","",IF(EDATE(サマリ!$B$2,1)&gt;$E20,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E20,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E20,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="10" t="n"/>
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="6" t="n"/>
-      <c r="L20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -1342,17 +1318,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
-      <c r="H21" s="6">
-        <f>IF($G21="","",IF(EDATE(サマリ!$B$2,1)&gt;$G21,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G21,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G21,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I21" s="6" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="6">
+        <f>IF($E21="","",IF(EDATE(サマリ!$B$2,1)&gt;$E21,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E21,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E21,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="10" t="n"/>
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
-      <c r="L21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -1371,17 +1346,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
-      <c r="H22" s="6">
-        <f>IF($G22="","",IF(EDATE(サマリ!$B$2,1)&gt;$G22,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G22,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G22,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I22" s="6" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="6">
+        <f>IF($E22="","",IF(EDATE(サマリ!$B$2,1)&gt;$E22,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E22,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E22,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="10" t="n"/>
       <c r="J22" s="6" t="n"/>
       <c r="K22" s="6" t="n"/>
-      <c r="L22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -1400,17 +1374,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="10" t="n"/>
-      <c r="H23" s="6">
-        <f>IF($G23="","",IF(EDATE(サマリ!$B$2,1)&gt;$G23,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G23,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G23,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I23" s="6" t="n"/>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="6">
+        <f>IF($E23="","",IF(EDATE(サマリ!$B$2,1)&gt;$E23,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E23,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E23,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="10" t="n"/>
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
-      <c r="L23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1429,17 +1402,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
-      <c r="H24" s="6">
-        <f>IF($G24="","",IF(EDATE(サマリ!$B$2,1)&gt;$G24,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G24,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G24,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I24" s="6" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="6">
+        <f>IF($E24="","",IF(EDATE(サマリ!$B$2,1)&gt;$E24,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E24,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E24,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="10" t="n"/>
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="6" t="n"/>
-      <c r="L24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -1458,17 +1430,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="10" t="n"/>
-      <c r="G25" s="10" t="n"/>
-      <c r="H25" s="6">
-        <f>IF($G25="","",IF(EDATE(サマリ!$B$2,1)&gt;$G25,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G25,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G25,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I25" s="6" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="6">
+        <f>IF($E25="","",IF(EDATE(サマリ!$B$2,1)&gt;$E25,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E25,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E25,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
+      <c r="I25" s="10" t="n"/>
       <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -1487,17 +1458,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
-      <c r="H26" s="6">
-        <f>IF($G26="","",IF(EDATE(サマリ!$B$2,1)&gt;$G26,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G26,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G26,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I26" s="6" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="6">
+        <f>IF($E26="","",IF(EDATE(サマリ!$B$2,1)&gt;$E26,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E26,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E26,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+      <c r="I26" s="10" t="n"/>
       <c r="J26" s="6" t="n"/>
       <c r="K26" s="6" t="n"/>
-      <c r="L26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -1516,17 +1486,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="10" t="n"/>
-      <c r="G27" s="10" t="n"/>
-      <c r="H27" s="6">
-        <f>IF($G27="","",IF(EDATE(サマリ!$B$2,1)&gt;$G27,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G27,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G27,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I27" s="6" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="6">
+        <f>IF($E27="","",IF(EDATE(サマリ!$B$2,1)&gt;$E27,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E27,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E27,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+      <c r="I27" s="10" t="n"/>
       <c r="J27" s="6" t="n"/>
       <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -1545,17 +1514,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="10" t="n"/>
-      <c r="H28" s="6">
-        <f>IF($G28="","",IF(EDATE(サマリ!$B$2,1)&gt;$G28,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G28,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G28,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I28" s="6" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="6">
+        <f>IF($E28="","",IF(EDATE(サマリ!$B$2,1)&gt;$E28,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E28,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E28,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
+      <c r="I28" s="10" t="n"/>
       <c r="J28" s="6" t="n"/>
       <c r="K28" s="6" t="n"/>
-      <c r="L28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -1574,17 +1542,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="10" t="n"/>
-      <c r="H29" s="6">
-        <f>IF($G29="","",IF(EDATE(サマリ!$B$2,1)&gt;$G29,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G29,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G29,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I29" s="6" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="6">
+        <f>IF($E29="","",IF(EDATE(サマリ!$B$2,1)&gt;$E29,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E29,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E29,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="6" t="n"/>
+      <c r="I29" s="10" t="n"/>
       <c r="J29" s="6" t="n"/>
       <c r="K29" s="6" t="n"/>
-      <c r="L29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -1603,17 +1570,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
-      <c r="H30" s="6">
-        <f>IF($G30="","",IF(EDATE(サマリ!$B$2,1)&gt;$G30,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G30,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G30,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I30" s="6" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="6">
+        <f>IF($E30="","",IF(EDATE(サマリ!$B$2,1)&gt;$E30,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E30,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E30,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="6" t="n"/>
+      <c r="I30" s="10" t="n"/>
       <c r="J30" s="6" t="n"/>
       <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -1632,17 +1598,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="10" t="n"/>
-      <c r="G31" s="10" t="n"/>
-      <c r="H31" s="6">
-        <f>IF($G31="","",IF(EDATE(サマリ!$B$2,1)&gt;$G31,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G31,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G31,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I31" s="6" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="6">
+        <f>IF($E31="","",IF(EDATE(サマリ!$B$2,1)&gt;$E31,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E31,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E31,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
+      <c r="I31" s="10" t="n"/>
       <c r="J31" s="6" t="n"/>
       <c r="K31" s="6" t="n"/>
-      <c r="L31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -1661,17 +1626,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="10" t="n"/>
-      <c r="G32" s="10" t="n"/>
-      <c r="H32" s="6">
-        <f>IF($G32="","",IF(EDATE(サマリ!$B$2,1)&gt;$G32,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G32,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G32,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I32" s="6" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="6">
+        <f>IF($E32="","",IF(EDATE(サマリ!$B$2,1)&gt;$E32,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E32,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E32,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="6" t="n"/>
+      <c r="I32" s="10" t="n"/>
       <c r="J32" s="6" t="n"/>
       <c r="K32" s="6" t="n"/>
-      <c r="L32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -1690,17 +1654,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="10" t="n"/>
-      <c r="G33" s="10" t="n"/>
-      <c r="H33" s="6">
-        <f>IF($G33="","",IF(EDATE(サマリ!$B$2,1)&gt;$G33,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G33,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G33,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I33" s="6" t="n"/>
+      <c r="E33" s="10" t="n"/>
+      <c r="F33" s="6">
+        <f>IF($E33="","",IF(EDATE(サマリ!$B$2,1)&gt;$E33,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E33,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E33,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="6" t="n"/>
+      <c r="I33" s="10" t="n"/>
       <c r="J33" s="6" t="n"/>
       <c r="K33" s="6" t="n"/>
-      <c r="L33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -1719,17 +1682,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="10" t="n"/>
-      <c r="G34" s="10" t="n"/>
-      <c r="H34" s="6">
-        <f>IF($G34="","",IF(EDATE(サマリ!$B$2,1)&gt;$G34,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G34,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G34,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I34" s="6" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="6">
+        <f>IF($E34="","",IF(EDATE(サマリ!$B$2,1)&gt;$E34,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E34,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E34,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G34" s="6" t="n"/>
+      <c r="H34" s="6" t="n"/>
+      <c r="I34" s="10" t="n"/>
       <c r="J34" s="6" t="n"/>
       <c r="K34" s="6" t="n"/>
-      <c r="L34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -1748,17 +1710,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="10" t="n"/>
-      <c r="G35" s="10" t="n"/>
-      <c r="H35" s="6">
-        <f>IF($G35="","",IF(EDATE(サマリ!$B$2,1)&gt;$G35,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G35,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G35,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I35" s="6" t="n"/>
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="6">
+        <f>IF($E35="","",IF(EDATE(サマリ!$B$2,1)&gt;$E35,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E35,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E35,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="6" t="n"/>
+      <c r="I35" s="10" t="n"/>
       <c r="J35" s="6" t="n"/>
       <c r="K35" s="6" t="n"/>
-      <c r="L35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -1777,17 +1738,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E36" s="6" t="n"/>
-      <c r="F36" s="10" t="n"/>
-      <c r="G36" s="10" t="n"/>
-      <c r="H36" s="6">
-        <f>IF($G36="","",IF(EDATE(サマリ!$B$2,1)&gt;$G36,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G36,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G36,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I36" s="6" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="6">
+        <f>IF($E36="","",IF(EDATE(サマリ!$B$2,1)&gt;$E36,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E36,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E36,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="6" t="n"/>
+      <c r="I36" s="10" t="n"/>
       <c r="J36" s="6" t="n"/>
       <c r="K36" s="6" t="n"/>
-      <c r="L36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -1806,17 +1766,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="10" t="n"/>
-      <c r="G37" s="10" t="n"/>
-      <c r="H37" s="6">
-        <f>IF($G37="","",IF(EDATE(サマリ!$B$2,1)&gt;$G37,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G37,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G37,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I37" s="6" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="6">
+        <f>IF($E37="","",IF(EDATE(サマリ!$B$2,1)&gt;$E37,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E37,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E37,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="6" t="n"/>
+      <c r="I37" s="10" t="n"/>
       <c r="J37" s="6" t="n"/>
       <c r="K37" s="6" t="n"/>
-      <c r="L37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -1835,17 +1794,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="10" t="n"/>
-      <c r="G38" s="10" t="n"/>
-      <c r="H38" s="6">
-        <f>IF($G38="","",IF(EDATE(サマリ!$B$2,1)&gt;$G38,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G38,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G38,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I38" s="6" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="6">
+        <f>IF($E38="","",IF(EDATE(サマリ!$B$2,1)&gt;$E38,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E38,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E38,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="10" t="n"/>
       <c r="J38" s="6" t="n"/>
       <c r="K38" s="6" t="n"/>
-      <c r="L38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -1864,17 +1822,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="10" t="n"/>
-      <c r="G39" s="10" t="n"/>
-      <c r="H39" s="6">
-        <f>IF($G39="","",IF(EDATE(サマリ!$B$2,1)&gt;$G39,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G39,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G39,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I39" s="6" t="n"/>
+      <c r="E39" s="10" t="n"/>
+      <c r="F39" s="6">
+        <f>IF($E39="","",IF(EDATE(サマリ!$B$2,1)&gt;$E39,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E39,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E39,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="10" t="n"/>
       <c r="J39" s="6" t="n"/>
       <c r="K39" s="6" t="n"/>
-      <c r="L39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr"/>
@@ -1889,17 +1846,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E40" s="6" t="n"/>
-      <c r="F40" s="10" t="n"/>
-      <c r="G40" s="10" t="n"/>
-      <c r="H40" s="6">
-        <f>IF($G40="","",IF(EDATE(サマリ!$B$2,1)&gt;$G40,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G40,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G40,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I40" s="6" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="6">
+        <f>IF($E40="","",IF(EDATE(サマリ!$B$2,1)&gt;$E40,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E40,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E40,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G40" s="6" t="n"/>
+      <c r="H40" s="6" t="n"/>
+      <c r="I40" s="10" t="n"/>
       <c r="J40" s="6" t="n"/>
       <c r="K40" s="6" t="n"/>
-      <c r="L40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr"/>
@@ -1914,25 +1870,24 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="10" t="n"/>
-      <c r="G41" s="10" t="n"/>
-      <c r="H41" s="6">
-        <f>IF($G41="","",IF(EDATE(サマリ!$B$2,1)&gt;$G41,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G41,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G41,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I41" s="6" t="n"/>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="6">
+        <f>IF($E41="","",IF(EDATE(サマリ!$B$2,1)&gt;$E41,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E41,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E41,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="10" t="n"/>
       <c r="J41" s="6" t="n"/>
       <c r="K41" s="6" t="n"/>
-      <c r="L41" s="6" t="n"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A4:L41">
+  <conditionalFormatting sqref="A4:K41">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$H4="期限切れ"</formula>
+      <formula>$F4="期限切れ"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$H4="来月期限"</formula>
+      <formula>$F4="来月期限"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C41">
@@ -1940,11 +1895,8 @@
       <formula>ISBLANK($C4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation sqref="J4:J41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=設定!$A$2:$A$11</formula1>
-    </dataValidation>
-    <dataValidation sqref="K4:K41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1回目完了,ダブルチェック完了"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1958,21 +1910,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:K90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2016,40 +1967,35 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
+          <t>期限日</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>期限区分(自動)</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>期限量</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
           <t>期限切れ量</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>期限切れ日</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>期限日</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>期限区分(自動)</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>期限量</t>
-        </is>
-      </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>入力者</t>
+          <t>チェック</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>チェック</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
@@ -2072,17 +2018,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="6">
-        <f>IF($G4="","",IF(EDATE(サマリ!$B$2,1)&gt;$G4,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G4,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G4,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I4" s="6" t="n"/>
+      <c r="E4" s="10" t="n"/>
+      <c r="F4" s="6">
+        <f>IF($E4="","",IF(EDATE(サマリ!$B$2,1)&gt;$E4,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E4,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E4,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="10" t="n"/>
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2101,17 +2046,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="6">
-        <f>IF($G5="","",IF(EDATE(サマリ!$B$2,1)&gt;$G5,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G5,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G5,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I5" s="6" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="6">
+        <f>IF($E5="","",IF(EDATE(サマリ!$B$2,1)&gt;$E5,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E5,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E5,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="10" t="n"/>
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="6" t="n"/>
-      <c r="L5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -2130,17 +2074,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="6">
-        <f>IF($G6="","",IF(EDATE(サマリ!$B$2,1)&gt;$G6,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G6,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G6,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I6" s="6" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="6">
+        <f>IF($E6="","",IF(EDATE(サマリ!$B$2,1)&gt;$E6,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E6,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E6,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="10" t="n"/>
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2159,17 +2102,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="6">
-        <f>IF($G7="","",IF(EDATE(サマリ!$B$2,1)&gt;$G7,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G7,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G7,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I7" s="6" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="6">
+        <f>IF($E7="","",IF(EDATE(サマリ!$B$2,1)&gt;$E7,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E7,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E7,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="10" t="n"/>
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
-      <c r="L7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2188,17 +2130,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="6">
-        <f>IF($G8="","",IF(EDATE(サマリ!$B$2,1)&gt;$G8,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G8,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G8,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I8" s="6" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="6">
+        <f>IF($E8="","",IF(EDATE(サマリ!$B$2,1)&gt;$E8,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E8,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E8,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="10" t="n"/>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
-      <c r="L8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2217,17 +2158,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="6">
-        <f>IF($G9="","",IF(EDATE(サマリ!$B$2,1)&gt;$G9,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G9,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G9,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I9" s="6" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="6">
+        <f>IF($E9="","",IF(EDATE(サマリ!$B$2,1)&gt;$E9,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E9,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E9,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="10" t="n"/>
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="6" t="n"/>
-      <c r="L9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -2246,17 +2186,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="6">
-        <f>IF($G10="","",IF(EDATE(サマリ!$B$2,1)&gt;$G10,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G10,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G10,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I10" s="6" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="6">
+        <f>IF($E10="","",IF(EDATE(サマリ!$B$2,1)&gt;$E10,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E10,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E10,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="10" t="n"/>
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
-      <c r="L10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -2275,17 +2214,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
-      <c r="H11" s="6">
-        <f>IF($G11="","",IF(EDATE(サマリ!$B$2,1)&gt;$G11,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G11,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G11,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I11" s="6" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="6">
+        <f>IF($E11="","",IF(EDATE(サマリ!$B$2,1)&gt;$E11,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E11,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E11,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="10" t="n"/>
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
-      <c r="L11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -2304,17 +2242,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="6">
-        <f>IF($G12="","",IF(EDATE(サマリ!$B$2,1)&gt;$G12,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G12,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G12,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I12" s="6" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="6">
+        <f>IF($E12="","",IF(EDATE(サマリ!$B$2,1)&gt;$E12,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E12,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E12,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="10" t="n"/>
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
-      <c r="L12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -2333,17 +2270,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
-      <c r="H13" s="6">
-        <f>IF($G13="","",IF(EDATE(サマリ!$B$2,1)&gt;$G13,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G13,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G13,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I13" s="6" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="6">
+        <f>IF($E13="","",IF(EDATE(サマリ!$B$2,1)&gt;$E13,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E13,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E13,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="10" t="n"/>
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
-      <c r="L13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -2362,17 +2298,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="6">
-        <f>IF($G14="","",IF(EDATE(サマリ!$B$2,1)&gt;$G14,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G14,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G14,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I14" s="6" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="6">
+        <f>IF($E14="","",IF(EDATE(サマリ!$B$2,1)&gt;$E14,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E14,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E14,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="10" t="n"/>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
-      <c r="L14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -2391,17 +2326,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
-      <c r="H15" s="6">
-        <f>IF($G15="","",IF(EDATE(サマリ!$B$2,1)&gt;$G15,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G15,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G15,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I15" s="6" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="6">
+        <f>IF($E15="","",IF(EDATE(サマリ!$B$2,1)&gt;$E15,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E15,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E15,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="10" t="n"/>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
-      <c r="L15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -2420,17 +2354,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="6">
-        <f>IF($G16="","",IF(EDATE(サマリ!$B$2,1)&gt;$G16,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G16,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G16,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I16" s="6" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="6">
+        <f>IF($E16="","",IF(EDATE(サマリ!$B$2,1)&gt;$E16,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E16,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E16,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="10" t="n"/>
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
-      <c r="L16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -2449,17 +2382,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
-      <c r="H17" s="6">
-        <f>IF($G17="","",IF(EDATE(サマリ!$B$2,1)&gt;$G17,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G17,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G17,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I17" s="6" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="6">
+        <f>IF($E17="","",IF(EDATE(サマリ!$B$2,1)&gt;$E17,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E17,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E17,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="10" t="n"/>
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
-      <c r="L17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -2478,17 +2410,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="6">
-        <f>IF($G18="","",IF(EDATE(サマリ!$B$2,1)&gt;$G18,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G18,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G18,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I18" s="6" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="6">
+        <f>IF($E18="","",IF(EDATE(サマリ!$B$2,1)&gt;$E18,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E18,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E18,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="10" t="n"/>
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
-      <c r="L18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -2507,17 +2438,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="6">
-        <f>IF($G19="","",IF(EDATE(サマリ!$B$2,1)&gt;$G19,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G19,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G19,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I19" s="6" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="6">
+        <f>IF($E19="","",IF(EDATE(サマリ!$B$2,1)&gt;$E19,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E19,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E19,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="10" t="n"/>
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
-      <c r="L19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -2536,17 +2466,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="6">
-        <f>IF($G20="","",IF(EDATE(サマリ!$B$2,1)&gt;$G20,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G20,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G20,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I20" s="6" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="6">
+        <f>IF($E20="","",IF(EDATE(サマリ!$B$2,1)&gt;$E20,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E20,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E20,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="10" t="n"/>
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="6" t="n"/>
-      <c r="L20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -2565,17 +2494,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
-      <c r="H21" s="6">
-        <f>IF($G21="","",IF(EDATE(サマリ!$B$2,1)&gt;$G21,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G21,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G21,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I21" s="6" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="6">
+        <f>IF($E21="","",IF(EDATE(サマリ!$B$2,1)&gt;$E21,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E21,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E21,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="10" t="n"/>
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
-      <c r="L21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -2594,17 +2522,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
-      <c r="H22" s="6">
-        <f>IF($G22="","",IF(EDATE(サマリ!$B$2,1)&gt;$G22,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G22,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G22,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I22" s="6" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="6">
+        <f>IF($E22="","",IF(EDATE(サマリ!$B$2,1)&gt;$E22,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E22,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E22,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="10" t="n"/>
       <c r="J22" s="6" t="n"/>
       <c r="K22" s="6" t="n"/>
-      <c r="L22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -2623,17 +2550,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="10" t="n"/>
-      <c r="H23" s="6">
-        <f>IF($G23="","",IF(EDATE(サマリ!$B$2,1)&gt;$G23,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G23,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G23,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I23" s="6" t="n"/>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="6">
+        <f>IF($E23="","",IF(EDATE(サマリ!$B$2,1)&gt;$E23,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E23,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E23,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="10" t="n"/>
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
-      <c r="L23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -2652,17 +2578,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
-      <c r="H24" s="6">
-        <f>IF($G24="","",IF(EDATE(サマリ!$B$2,1)&gt;$G24,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G24,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G24,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I24" s="6" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="6">
+        <f>IF($E24="","",IF(EDATE(サマリ!$B$2,1)&gt;$E24,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E24,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E24,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="10" t="n"/>
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="6" t="n"/>
-      <c r="L24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -2681,17 +2606,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="10" t="n"/>
-      <c r="G25" s="10" t="n"/>
-      <c r="H25" s="6">
-        <f>IF($G25="","",IF(EDATE(サマリ!$B$2,1)&gt;$G25,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G25,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G25,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I25" s="6" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="6">
+        <f>IF($E25="","",IF(EDATE(サマリ!$B$2,1)&gt;$E25,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E25,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E25,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
+      <c r="I25" s="10" t="n"/>
       <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -2710,17 +2634,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
-      <c r="H26" s="6">
-        <f>IF($G26="","",IF(EDATE(サマリ!$B$2,1)&gt;$G26,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G26,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G26,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I26" s="6" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="6">
+        <f>IF($E26="","",IF(EDATE(サマリ!$B$2,1)&gt;$E26,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E26,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E26,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+      <c r="I26" s="10" t="n"/>
       <c r="J26" s="6" t="n"/>
       <c r="K26" s="6" t="n"/>
-      <c r="L26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -2739,17 +2662,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="10" t="n"/>
-      <c r="G27" s="10" t="n"/>
-      <c r="H27" s="6">
-        <f>IF($G27="","",IF(EDATE(サマリ!$B$2,1)&gt;$G27,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G27,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G27,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I27" s="6" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="6">
+        <f>IF($E27="","",IF(EDATE(サマリ!$B$2,1)&gt;$E27,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E27,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E27,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+      <c r="I27" s="10" t="n"/>
       <c r="J27" s="6" t="n"/>
       <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -2768,17 +2690,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="10" t="n"/>
-      <c r="H28" s="6">
-        <f>IF($G28="","",IF(EDATE(サマリ!$B$2,1)&gt;$G28,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G28,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G28,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I28" s="6" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="6">
+        <f>IF($E28="","",IF(EDATE(サマリ!$B$2,1)&gt;$E28,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E28,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E28,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
+      <c r="I28" s="10" t="n"/>
       <c r="J28" s="6" t="n"/>
       <c r="K28" s="6" t="n"/>
-      <c r="L28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -2797,17 +2718,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="10" t="n"/>
-      <c r="H29" s="6">
-        <f>IF($G29="","",IF(EDATE(サマリ!$B$2,1)&gt;$G29,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G29,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G29,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I29" s="6" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="6">
+        <f>IF($E29="","",IF(EDATE(サマリ!$B$2,1)&gt;$E29,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E29,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E29,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="6" t="n"/>
+      <c r="I29" s="10" t="n"/>
       <c r="J29" s="6" t="n"/>
       <c r="K29" s="6" t="n"/>
-      <c r="L29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -2826,17 +2746,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
-      <c r="H30" s="6">
-        <f>IF($G30="","",IF(EDATE(サマリ!$B$2,1)&gt;$G30,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G30,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G30,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I30" s="6" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="6">
+        <f>IF($E30="","",IF(EDATE(サマリ!$B$2,1)&gt;$E30,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E30,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E30,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="6" t="n"/>
+      <c r="I30" s="10" t="n"/>
       <c r="J30" s="6" t="n"/>
       <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -2855,17 +2774,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="10" t="n"/>
-      <c r="G31" s="10" t="n"/>
-      <c r="H31" s="6">
-        <f>IF($G31="","",IF(EDATE(サマリ!$B$2,1)&gt;$G31,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G31,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G31,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I31" s="6" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="6">
+        <f>IF($E31="","",IF(EDATE(サマリ!$B$2,1)&gt;$E31,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E31,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E31,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
+      <c r="I31" s="10" t="n"/>
       <c r="J31" s="6" t="n"/>
       <c r="K31" s="6" t="n"/>
-      <c r="L31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -2884,17 +2802,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="10" t="n"/>
-      <c r="G32" s="10" t="n"/>
-      <c r="H32" s="6">
-        <f>IF($G32="","",IF(EDATE(サマリ!$B$2,1)&gt;$G32,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G32,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G32,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I32" s="6" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="6">
+        <f>IF($E32="","",IF(EDATE(サマリ!$B$2,1)&gt;$E32,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E32,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E32,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="6" t="n"/>
+      <c r="I32" s="10" t="n"/>
       <c r="J32" s="6" t="n"/>
       <c r="K32" s="6" t="n"/>
-      <c r="L32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -2913,17 +2830,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="10" t="n"/>
-      <c r="G33" s="10" t="n"/>
-      <c r="H33" s="6">
-        <f>IF($G33="","",IF(EDATE(サマリ!$B$2,1)&gt;$G33,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G33,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G33,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I33" s="6" t="n"/>
+      <c r="E33" s="10" t="n"/>
+      <c r="F33" s="6">
+        <f>IF($E33="","",IF(EDATE(サマリ!$B$2,1)&gt;$E33,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E33,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E33,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="6" t="n"/>
+      <c r="I33" s="10" t="n"/>
       <c r="J33" s="6" t="n"/>
       <c r="K33" s="6" t="n"/>
-      <c r="L33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -2942,17 +2858,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="10" t="n"/>
-      <c r="G34" s="10" t="n"/>
-      <c r="H34" s="6">
-        <f>IF($G34="","",IF(EDATE(サマリ!$B$2,1)&gt;$G34,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G34,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G34,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I34" s="6" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="6">
+        <f>IF($E34="","",IF(EDATE(サマリ!$B$2,1)&gt;$E34,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E34,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E34,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G34" s="6" t="n"/>
+      <c r="H34" s="6" t="n"/>
+      <c r="I34" s="10" t="n"/>
       <c r="J34" s="6" t="n"/>
       <c r="K34" s="6" t="n"/>
-      <c r="L34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -2971,17 +2886,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="10" t="n"/>
-      <c r="G35" s="10" t="n"/>
-      <c r="H35" s="6">
-        <f>IF($G35="","",IF(EDATE(サマリ!$B$2,1)&gt;$G35,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G35,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G35,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I35" s="6" t="n"/>
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="6">
+        <f>IF($E35="","",IF(EDATE(サマリ!$B$2,1)&gt;$E35,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E35,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E35,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="6" t="n"/>
+      <c r="I35" s="10" t="n"/>
       <c r="J35" s="6" t="n"/>
       <c r="K35" s="6" t="n"/>
-      <c r="L35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -3000,17 +2914,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E36" s="6" t="n"/>
-      <c r="F36" s="10" t="n"/>
-      <c r="G36" s="10" t="n"/>
-      <c r="H36" s="6">
-        <f>IF($G36="","",IF(EDATE(サマリ!$B$2,1)&gt;$G36,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G36,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G36,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I36" s="6" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="6">
+        <f>IF($E36="","",IF(EDATE(サマリ!$B$2,1)&gt;$E36,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E36,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E36,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="6" t="n"/>
+      <c r="I36" s="10" t="n"/>
       <c r="J36" s="6" t="n"/>
       <c r="K36" s="6" t="n"/>
-      <c r="L36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -3029,17 +2942,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="10" t="n"/>
-      <c r="G37" s="10" t="n"/>
-      <c r="H37" s="6">
-        <f>IF($G37="","",IF(EDATE(サマリ!$B$2,1)&gt;$G37,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G37,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G37,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I37" s="6" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="6">
+        <f>IF($E37="","",IF(EDATE(サマリ!$B$2,1)&gt;$E37,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E37,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E37,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="6" t="n"/>
+      <c r="I37" s="10" t="n"/>
       <c r="J37" s="6" t="n"/>
       <c r="K37" s="6" t="n"/>
-      <c r="L37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -3058,17 +2970,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="10" t="n"/>
-      <c r="G38" s="10" t="n"/>
-      <c r="H38" s="6">
-        <f>IF($G38="","",IF(EDATE(サマリ!$B$2,1)&gt;$G38,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G38,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G38,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I38" s="6" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="6">
+        <f>IF($E38="","",IF(EDATE(サマリ!$B$2,1)&gt;$E38,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E38,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E38,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="10" t="n"/>
       <c r="J38" s="6" t="n"/>
       <c r="K38" s="6" t="n"/>
-      <c r="L38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -3087,17 +2998,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="10" t="n"/>
-      <c r="G39" s="10" t="n"/>
-      <c r="H39" s="6">
-        <f>IF($G39="","",IF(EDATE(サマリ!$B$2,1)&gt;$G39,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G39,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G39,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I39" s="6" t="n"/>
+      <c r="E39" s="10" t="n"/>
+      <c r="F39" s="6">
+        <f>IF($E39="","",IF(EDATE(サマリ!$B$2,1)&gt;$E39,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E39,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E39,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="10" t="n"/>
       <c r="J39" s="6" t="n"/>
       <c r="K39" s="6" t="n"/>
-      <c r="L39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -3116,17 +3026,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E40" s="6" t="n"/>
-      <c r="F40" s="10" t="n"/>
-      <c r="G40" s="10" t="n"/>
-      <c r="H40" s="6">
-        <f>IF($G40="","",IF(EDATE(サマリ!$B$2,1)&gt;$G40,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G40,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G40,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I40" s="6" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="6">
+        <f>IF($E40="","",IF(EDATE(サマリ!$B$2,1)&gt;$E40,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E40,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E40,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G40" s="6" t="n"/>
+      <c r="H40" s="6" t="n"/>
+      <c r="I40" s="10" t="n"/>
       <c r="J40" s="6" t="n"/>
       <c r="K40" s="6" t="n"/>
-      <c r="L40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -3145,17 +3054,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="10" t="n"/>
-      <c r="G41" s="10" t="n"/>
-      <c r="H41" s="6">
-        <f>IF($G41="","",IF(EDATE(サマリ!$B$2,1)&gt;$G41,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G41,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G41,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I41" s="6" t="n"/>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="6">
+        <f>IF($E41="","",IF(EDATE(サマリ!$B$2,1)&gt;$E41,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E41,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E41,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="10" t="n"/>
       <c r="J41" s="6" t="n"/>
       <c r="K41" s="6" t="n"/>
-      <c r="L41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -3174,17 +3082,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E42" s="6" t="n"/>
-      <c r="F42" s="10" t="n"/>
-      <c r="G42" s="10" t="n"/>
-      <c r="H42" s="6">
-        <f>IF($G42="","",IF(EDATE(サマリ!$B$2,1)&gt;$G42,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G42,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G42,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I42" s="6" t="n"/>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="6">
+        <f>IF($E42="","",IF(EDATE(サマリ!$B$2,1)&gt;$E42,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E42,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E42,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="6" t="n"/>
+      <c r="I42" s="10" t="n"/>
       <c r="J42" s="6" t="n"/>
       <c r="K42" s="6" t="n"/>
-      <c r="L42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -3203,17 +3110,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E43" s="6" t="n"/>
-      <c r="F43" s="10" t="n"/>
-      <c r="G43" s="10" t="n"/>
-      <c r="H43" s="6">
-        <f>IF($G43="","",IF(EDATE(サマリ!$B$2,1)&gt;$G43,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G43,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G43,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I43" s="6" t="n"/>
+      <c r="E43" s="10" t="n"/>
+      <c r="F43" s="6">
+        <f>IF($E43="","",IF(EDATE(サマリ!$B$2,1)&gt;$E43,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E43,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E43,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G43" s="6" t="n"/>
+      <c r="H43" s="6" t="n"/>
+      <c r="I43" s="10" t="n"/>
       <c r="J43" s="6" t="n"/>
       <c r="K43" s="6" t="n"/>
-      <c r="L43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -3232,17 +3138,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E44" s="6" t="n"/>
-      <c r="F44" s="10" t="n"/>
-      <c r="G44" s="10" t="n"/>
-      <c r="H44" s="6">
-        <f>IF($G44="","",IF(EDATE(サマリ!$B$2,1)&gt;$G44,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G44,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G44,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I44" s="6" t="n"/>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="6">
+        <f>IF($E44="","",IF(EDATE(サマリ!$B$2,1)&gt;$E44,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E44,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E44,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G44" s="6" t="n"/>
+      <c r="H44" s="6" t="n"/>
+      <c r="I44" s="10" t="n"/>
       <c r="J44" s="6" t="n"/>
       <c r="K44" s="6" t="n"/>
-      <c r="L44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -3261,17 +3166,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E45" s="6" t="n"/>
-      <c r="F45" s="10" t="n"/>
-      <c r="G45" s="10" t="n"/>
-      <c r="H45" s="6">
-        <f>IF($G45="","",IF(EDATE(サマリ!$B$2,1)&gt;$G45,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G45,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G45,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I45" s="6" t="n"/>
+      <c r="E45" s="10" t="n"/>
+      <c r="F45" s="6">
+        <f>IF($E45="","",IF(EDATE(サマリ!$B$2,1)&gt;$E45,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E45,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E45,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G45" s="6" t="n"/>
+      <c r="H45" s="6" t="n"/>
+      <c r="I45" s="10" t="n"/>
       <c r="J45" s="6" t="n"/>
       <c r="K45" s="6" t="n"/>
-      <c r="L45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -3290,17 +3194,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E46" s="6" t="n"/>
-      <c r="F46" s="10" t="n"/>
-      <c r="G46" s="10" t="n"/>
-      <c r="H46" s="6">
-        <f>IF($G46="","",IF(EDATE(サマリ!$B$2,1)&gt;$G46,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G46,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G46,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I46" s="6" t="n"/>
+      <c r="E46" s="10" t="n"/>
+      <c r="F46" s="6">
+        <f>IF($E46="","",IF(EDATE(サマリ!$B$2,1)&gt;$E46,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E46,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E46,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="6" t="n"/>
+      <c r="I46" s="10" t="n"/>
       <c r="J46" s="6" t="n"/>
       <c r="K46" s="6" t="n"/>
-      <c r="L46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -3319,17 +3222,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E47" s="6" t="n"/>
-      <c r="F47" s="10" t="n"/>
-      <c r="G47" s="10" t="n"/>
-      <c r="H47" s="6">
-        <f>IF($G47="","",IF(EDATE(サマリ!$B$2,1)&gt;$G47,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G47,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G47,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I47" s="6" t="n"/>
+      <c r="E47" s="10" t="n"/>
+      <c r="F47" s="6">
+        <f>IF($E47="","",IF(EDATE(サマリ!$B$2,1)&gt;$E47,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E47,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E47,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="6" t="n"/>
+      <c r="I47" s="10" t="n"/>
       <c r="J47" s="6" t="n"/>
       <c r="K47" s="6" t="n"/>
-      <c r="L47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -3348,17 +3250,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E48" s="6" t="n"/>
-      <c r="F48" s="10" t="n"/>
-      <c r="G48" s="10" t="n"/>
-      <c r="H48" s="6">
-        <f>IF($G48="","",IF(EDATE(サマリ!$B$2,1)&gt;$G48,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G48,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G48,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I48" s="6" t="n"/>
+      <c r="E48" s="10" t="n"/>
+      <c r="F48" s="6">
+        <f>IF($E48="","",IF(EDATE(サマリ!$B$2,1)&gt;$E48,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E48,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E48,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G48" s="6" t="n"/>
+      <c r="H48" s="6" t="n"/>
+      <c r="I48" s="10" t="n"/>
       <c r="J48" s="6" t="n"/>
       <c r="K48" s="6" t="n"/>
-      <c r="L48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -3377,17 +3278,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E49" s="6" t="n"/>
-      <c r="F49" s="10" t="n"/>
-      <c r="G49" s="10" t="n"/>
-      <c r="H49" s="6">
-        <f>IF($G49="","",IF(EDATE(サマリ!$B$2,1)&gt;$G49,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G49,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G49,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I49" s="6" t="n"/>
+      <c r="E49" s="10" t="n"/>
+      <c r="F49" s="6">
+        <f>IF($E49="","",IF(EDATE(サマリ!$B$2,1)&gt;$E49,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E49,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E49,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="6" t="n"/>
+      <c r="I49" s="10" t="n"/>
       <c r="J49" s="6" t="n"/>
       <c r="K49" s="6" t="n"/>
-      <c r="L49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
@@ -3406,17 +3306,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E50" s="6" t="n"/>
-      <c r="F50" s="10" t="n"/>
-      <c r="G50" s="10" t="n"/>
-      <c r="H50" s="6">
-        <f>IF($G50="","",IF(EDATE(サマリ!$B$2,1)&gt;$G50,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G50,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G50,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I50" s="6" t="n"/>
+      <c r="E50" s="10" t="n"/>
+      <c r="F50" s="6">
+        <f>IF($E50="","",IF(EDATE(サマリ!$B$2,1)&gt;$E50,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E50,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E50,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G50" s="6" t="n"/>
+      <c r="H50" s="6" t="n"/>
+      <c r="I50" s="10" t="n"/>
       <c r="J50" s="6" t="n"/>
       <c r="K50" s="6" t="n"/>
-      <c r="L50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -3435,17 +3334,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E51" s="6" t="n"/>
-      <c r="F51" s="10" t="n"/>
-      <c r="G51" s="10" t="n"/>
-      <c r="H51" s="6">
-        <f>IF($G51="","",IF(EDATE(サマリ!$B$2,1)&gt;$G51,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G51,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G51,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I51" s="6" t="n"/>
+      <c r="E51" s="10" t="n"/>
+      <c r="F51" s="6">
+        <f>IF($E51="","",IF(EDATE(サマリ!$B$2,1)&gt;$E51,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E51,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E51,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G51" s="6" t="n"/>
+      <c r="H51" s="6" t="n"/>
+      <c r="I51" s="10" t="n"/>
       <c r="J51" s="6" t="n"/>
       <c r="K51" s="6" t="n"/>
-      <c r="L51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -3464,17 +3362,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E52" s="6" t="n"/>
-      <c r="F52" s="10" t="n"/>
-      <c r="G52" s="10" t="n"/>
-      <c r="H52" s="6">
-        <f>IF($G52="","",IF(EDATE(サマリ!$B$2,1)&gt;$G52,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G52,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G52,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I52" s="6" t="n"/>
+      <c r="E52" s="10" t="n"/>
+      <c r="F52" s="6">
+        <f>IF($E52="","",IF(EDATE(サマリ!$B$2,1)&gt;$E52,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E52,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E52,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G52" s="6" t="n"/>
+      <c r="H52" s="6" t="n"/>
+      <c r="I52" s="10" t="n"/>
       <c r="J52" s="6" t="n"/>
       <c r="K52" s="6" t="n"/>
-      <c r="L52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -3493,17 +3390,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E53" s="6" t="n"/>
-      <c r="F53" s="10" t="n"/>
-      <c r="G53" s="10" t="n"/>
-      <c r="H53" s="6">
-        <f>IF($G53="","",IF(EDATE(サマリ!$B$2,1)&gt;$G53,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G53,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G53,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I53" s="6" t="n"/>
+      <c r="E53" s="10" t="n"/>
+      <c r="F53" s="6">
+        <f>IF($E53="","",IF(EDATE(サマリ!$B$2,1)&gt;$E53,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E53,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E53,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G53" s="6" t="n"/>
+      <c r="H53" s="6" t="n"/>
+      <c r="I53" s="10" t="n"/>
       <c r="J53" s="6" t="n"/>
       <c r="K53" s="6" t="n"/>
-      <c r="L53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
@@ -3522,17 +3418,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E54" s="6" t="n"/>
-      <c r="F54" s="10" t="n"/>
-      <c r="G54" s="10" t="n"/>
-      <c r="H54" s="6">
-        <f>IF($G54="","",IF(EDATE(サマリ!$B$2,1)&gt;$G54,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G54,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G54,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I54" s="6" t="n"/>
+      <c r="E54" s="10" t="n"/>
+      <c r="F54" s="6">
+        <f>IF($E54="","",IF(EDATE(サマリ!$B$2,1)&gt;$E54,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E54,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E54,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G54" s="6" t="n"/>
+      <c r="H54" s="6" t="n"/>
+      <c r="I54" s="10" t="n"/>
       <c r="J54" s="6" t="n"/>
       <c r="K54" s="6" t="n"/>
-      <c r="L54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -3551,17 +3446,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E55" s="6" t="n"/>
-      <c r="F55" s="10" t="n"/>
-      <c r="G55" s="10" t="n"/>
-      <c r="H55" s="6">
-        <f>IF($G55="","",IF(EDATE(サマリ!$B$2,1)&gt;$G55,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G55,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G55,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I55" s="6" t="n"/>
+      <c r="E55" s="10" t="n"/>
+      <c r="F55" s="6">
+        <f>IF($E55="","",IF(EDATE(サマリ!$B$2,1)&gt;$E55,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E55,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E55,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G55" s="6" t="n"/>
+      <c r="H55" s="6" t="n"/>
+      <c r="I55" s="10" t="n"/>
       <c r="J55" s="6" t="n"/>
       <c r="K55" s="6" t="n"/>
-      <c r="L55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -3580,17 +3474,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E56" s="6" t="n"/>
-      <c r="F56" s="10" t="n"/>
-      <c r="G56" s="10" t="n"/>
-      <c r="H56" s="6">
-        <f>IF($G56="","",IF(EDATE(サマリ!$B$2,1)&gt;$G56,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G56,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G56,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I56" s="6" t="n"/>
+      <c r="E56" s="10" t="n"/>
+      <c r="F56" s="6">
+        <f>IF($E56="","",IF(EDATE(サマリ!$B$2,1)&gt;$E56,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E56,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E56,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G56" s="6" t="n"/>
+      <c r="H56" s="6" t="n"/>
+      <c r="I56" s="10" t="n"/>
       <c r="J56" s="6" t="n"/>
       <c r="K56" s="6" t="n"/>
-      <c r="L56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -3609,17 +3502,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E57" s="6" t="n"/>
-      <c r="F57" s="10" t="n"/>
-      <c r="G57" s="10" t="n"/>
-      <c r="H57" s="6">
-        <f>IF($G57="","",IF(EDATE(サマリ!$B$2,1)&gt;$G57,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G57,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G57,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I57" s="6" t="n"/>
+      <c r="E57" s="10" t="n"/>
+      <c r="F57" s="6">
+        <f>IF($E57="","",IF(EDATE(サマリ!$B$2,1)&gt;$E57,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E57,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E57,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G57" s="6" t="n"/>
+      <c r="H57" s="6" t="n"/>
+      <c r="I57" s="10" t="n"/>
       <c r="J57" s="6" t="n"/>
       <c r="K57" s="6" t="n"/>
-      <c r="L57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -3638,17 +3530,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E58" s="6" t="n"/>
-      <c r="F58" s="10" t="n"/>
-      <c r="G58" s="10" t="n"/>
-      <c r="H58" s="6">
-        <f>IF($G58="","",IF(EDATE(サマリ!$B$2,1)&gt;$G58,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G58,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G58,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I58" s="6" t="n"/>
+      <c r="E58" s="10" t="n"/>
+      <c r="F58" s="6">
+        <f>IF($E58="","",IF(EDATE(サマリ!$B$2,1)&gt;$E58,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E58,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E58,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G58" s="6" t="n"/>
+      <c r="H58" s="6" t="n"/>
+      <c r="I58" s="10" t="n"/>
       <c r="J58" s="6" t="n"/>
       <c r="K58" s="6" t="n"/>
-      <c r="L58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
@@ -3667,17 +3558,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E59" s="6" t="n"/>
-      <c r="F59" s="10" t="n"/>
-      <c r="G59" s="10" t="n"/>
-      <c r="H59" s="6">
-        <f>IF($G59="","",IF(EDATE(サマリ!$B$2,1)&gt;$G59,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G59,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G59,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I59" s="6" t="n"/>
+      <c r="E59" s="10" t="n"/>
+      <c r="F59" s="6">
+        <f>IF($E59="","",IF(EDATE(サマリ!$B$2,1)&gt;$E59,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E59,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E59,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G59" s="6" t="n"/>
+      <c r="H59" s="6" t="n"/>
+      <c r="I59" s="10" t="n"/>
       <c r="J59" s="6" t="n"/>
       <c r="K59" s="6" t="n"/>
-      <c r="L59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -3696,17 +3586,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E60" s="6" t="n"/>
-      <c r="F60" s="10" t="n"/>
-      <c r="G60" s="10" t="n"/>
-      <c r="H60" s="6">
-        <f>IF($G60="","",IF(EDATE(サマリ!$B$2,1)&gt;$G60,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G60,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G60,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I60" s="6" t="n"/>
+      <c r="E60" s="10" t="n"/>
+      <c r="F60" s="6">
+        <f>IF($E60="","",IF(EDATE(サマリ!$B$2,1)&gt;$E60,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E60,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E60,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G60" s="6" t="n"/>
+      <c r="H60" s="6" t="n"/>
+      <c r="I60" s="10" t="n"/>
       <c r="J60" s="6" t="n"/>
       <c r="K60" s="6" t="n"/>
-      <c r="L60" s="6" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
@@ -3725,17 +3614,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E61" s="6" t="n"/>
-      <c r="F61" s="10" t="n"/>
-      <c r="G61" s="10" t="n"/>
-      <c r="H61" s="6">
-        <f>IF($G61="","",IF(EDATE(サマリ!$B$2,1)&gt;$G61,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G61,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G61,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I61" s="6" t="n"/>
+      <c r="E61" s="10" t="n"/>
+      <c r="F61" s="6">
+        <f>IF($E61="","",IF(EDATE(サマリ!$B$2,1)&gt;$E61,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E61,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E61,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G61" s="6" t="n"/>
+      <c r="H61" s="6" t="n"/>
+      <c r="I61" s="10" t="n"/>
       <c r="J61" s="6" t="n"/>
       <c r="K61" s="6" t="n"/>
-      <c r="L61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
@@ -3754,17 +3642,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E62" s="6" t="n"/>
-      <c r="F62" s="10" t="n"/>
-      <c r="G62" s="10" t="n"/>
-      <c r="H62" s="6">
-        <f>IF($G62="","",IF(EDATE(サマリ!$B$2,1)&gt;$G62,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G62,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G62,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I62" s="6" t="n"/>
+      <c r="E62" s="10" t="n"/>
+      <c r="F62" s="6">
+        <f>IF($E62="","",IF(EDATE(サマリ!$B$2,1)&gt;$E62,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E62,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E62,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G62" s="6" t="n"/>
+      <c r="H62" s="6" t="n"/>
+      <c r="I62" s="10" t="n"/>
       <c r="J62" s="6" t="n"/>
       <c r="K62" s="6" t="n"/>
-      <c r="L62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
@@ -3783,17 +3670,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E63" s="6" t="n"/>
-      <c r="F63" s="10" t="n"/>
-      <c r="G63" s="10" t="n"/>
-      <c r="H63" s="6">
-        <f>IF($G63="","",IF(EDATE(サマリ!$B$2,1)&gt;$G63,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G63,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G63,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I63" s="6" t="n"/>
+      <c r="E63" s="10" t="n"/>
+      <c r="F63" s="6">
+        <f>IF($E63="","",IF(EDATE(サマリ!$B$2,1)&gt;$E63,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E63,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E63,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G63" s="6" t="n"/>
+      <c r="H63" s="6" t="n"/>
+      <c r="I63" s="10" t="n"/>
       <c r="J63" s="6" t="n"/>
       <c r="K63" s="6" t="n"/>
-      <c r="L63" s="6" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
@@ -3812,17 +3698,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E64" s="6" t="n"/>
-      <c r="F64" s="10" t="n"/>
-      <c r="G64" s="10" t="n"/>
-      <c r="H64" s="6">
-        <f>IF($G64="","",IF(EDATE(サマリ!$B$2,1)&gt;$G64,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G64,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G64,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I64" s="6" t="n"/>
+      <c r="E64" s="10" t="n"/>
+      <c r="F64" s="6">
+        <f>IF($E64="","",IF(EDATE(サマリ!$B$2,1)&gt;$E64,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E64,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E64,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G64" s="6" t="n"/>
+      <c r="H64" s="6" t="n"/>
+      <c r="I64" s="10" t="n"/>
       <c r="J64" s="6" t="n"/>
       <c r="K64" s="6" t="n"/>
-      <c r="L64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -3841,17 +3726,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E65" s="6" t="n"/>
-      <c r="F65" s="10" t="n"/>
-      <c r="G65" s="10" t="n"/>
-      <c r="H65" s="6">
-        <f>IF($G65="","",IF(EDATE(サマリ!$B$2,1)&gt;$G65,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G65,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G65,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I65" s="6" t="n"/>
+      <c r="E65" s="10" t="n"/>
+      <c r="F65" s="6">
+        <f>IF($E65="","",IF(EDATE(サマリ!$B$2,1)&gt;$E65,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E65,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E65,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G65" s="6" t="n"/>
+      <c r="H65" s="6" t="n"/>
+      <c r="I65" s="10" t="n"/>
       <c r="J65" s="6" t="n"/>
       <c r="K65" s="6" t="n"/>
-      <c r="L65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
@@ -3870,17 +3754,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E66" s="6" t="n"/>
-      <c r="F66" s="10" t="n"/>
-      <c r="G66" s="10" t="n"/>
-      <c r="H66" s="6">
-        <f>IF($G66="","",IF(EDATE(サマリ!$B$2,1)&gt;$G66,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G66,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G66,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I66" s="6" t="n"/>
+      <c r="E66" s="10" t="n"/>
+      <c r="F66" s="6">
+        <f>IF($E66="","",IF(EDATE(サマリ!$B$2,1)&gt;$E66,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E66,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E66,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G66" s="6" t="n"/>
+      <c r="H66" s="6" t="n"/>
+      <c r="I66" s="10" t="n"/>
       <c r="J66" s="6" t="n"/>
       <c r="K66" s="6" t="n"/>
-      <c r="L66" s="6" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
@@ -3899,17 +3782,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E67" s="6" t="n"/>
-      <c r="F67" s="10" t="n"/>
-      <c r="G67" s="10" t="n"/>
-      <c r="H67" s="6">
-        <f>IF($G67="","",IF(EDATE(サマリ!$B$2,1)&gt;$G67,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G67,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G67,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I67" s="6" t="n"/>
+      <c r="E67" s="10" t="n"/>
+      <c r="F67" s="6">
+        <f>IF($E67="","",IF(EDATE(サマリ!$B$2,1)&gt;$E67,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E67,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E67,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G67" s="6" t="n"/>
+      <c r="H67" s="6" t="n"/>
+      <c r="I67" s="10" t="n"/>
       <c r="J67" s="6" t="n"/>
       <c r="K67" s="6" t="n"/>
-      <c r="L67" s="6" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -3928,17 +3810,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E68" s="6" t="n"/>
-      <c r="F68" s="10" t="n"/>
-      <c r="G68" s="10" t="n"/>
-      <c r="H68" s="6">
-        <f>IF($G68="","",IF(EDATE(サマリ!$B$2,1)&gt;$G68,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G68,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G68,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I68" s="6" t="n"/>
+      <c r="E68" s="10" t="n"/>
+      <c r="F68" s="6">
+        <f>IF($E68="","",IF(EDATE(サマリ!$B$2,1)&gt;$E68,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E68,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E68,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G68" s="6" t="n"/>
+      <c r="H68" s="6" t="n"/>
+      <c r="I68" s="10" t="n"/>
       <c r="J68" s="6" t="n"/>
       <c r="K68" s="6" t="n"/>
-      <c r="L68" s="6" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -3957,17 +3838,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E69" s="6" t="n"/>
-      <c r="F69" s="10" t="n"/>
-      <c r="G69" s="10" t="n"/>
-      <c r="H69" s="6">
-        <f>IF($G69="","",IF(EDATE(サマリ!$B$2,1)&gt;$G69,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G69,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G69,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I69" s="6" t="n"/>
+      <c r="E69" s="10" t="n"/>
+      <c r="F69" s="6">
+        <f>IF($E69="","",IF(EDATE(サマリ!$B$2,1)&gt;$E69,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E69,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E69,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G69" s="6" t="n"/>
+      <c r="H69" s="6" t="n"/>
+      <c r="I69" s="10" t="n"/>
       <c r="J69" s="6" t="n"/>
       <c r="K69" s="6" t="n"/>
-      <c r="L69" s="6" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
@@ -3986,17 +3866,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E70" s="6" t="n"/>
-      <c r="F70" s="10" t="n"/>
-      <c r="G70" s="10" t="n"/>
-      <c r="H70" s="6">
-        <f>IF($G70="","",IF(EDATE(サマリ!$B$2,1)&gt;$G70,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G70,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G70,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I70" s="6" t="n"/>
+      <c r="E70" s="10" t="n"/>
+      <c r="F70" s="6">
+        <f>IF($E70="","",IF(EDATE(サマリ!$B$2,1)&gt;$E70,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E70,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E70,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G70" s="6" t="n"/>
+      <c r="H70" s="6" t="n"/>
+      <c r="I70" s="10" t="n"/>
       <c r="J70" s="6" t="n"/>
       <c r="K70" s="6" t="n"/>
-      <c r="L70" s="6" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
@@ -4015,17 +3894,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E71" s="6" t="n"/>
-      <c r="F71" s="10" t="n"/>
-      <c r="G71" s="10" t="n"/>
-      <c r="H71" s="6">
-        <f>IF($G71="","",IF(EDATE(サマリ!$B$2,1)&gt;$G71,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G71,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G71,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I71" s="6" t="n"/>
+      <c r="E71" s="10" t="n"/>
+      <c r="F71" s="6">
+        <f>IF($E71="","",IF(EDATE(サマリ!$B$2,1)&gt;$E71,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E71,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E71,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G71" s="6" t="n"/>
+      <c r="H71" s="6" t="n"/>
+      <c r="I71" s="10" t="n"/>
       <c r="J71" s="6" t="n"/>
       <c r="K71" s="6" t="n"/>
-      <c r="L71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -4044,17 +3922,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E72" s="6" t="n"/>
-      <c r="F72" s="10" t="n"/>
-      <c r="G72" s="10" t="n"/>
-      <c r="H72" s="6">
-        <f>IF($G72="","",IF(EDATE(サマリ!$B$2,1)&gt;$G72,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G72,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G72,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I72" s="6" t="n"/>
+      <c r="E72" s="10" t="n"/>
+      <c r="F72" s="6">
+        <f>IF($E72="","",IF(EDATE(サマリ!$B$2,1)&gt;$E72,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E72,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E72,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G72" s="6" t="n"/>
+      <c r="H72" s="6" t="n"/>
+      <c r="I72" s="10" t="n"/>
       <c r="J72" s="6" t="n"/>
       <c r="K72" s="6" t="n"/>
-      <c r="L72" s="6" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
@@ -4073,17 +3950,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E73" s="6" t="n"/>
-      <c r="F73" s="10" t="n"/>
-      <c r="G73" s="10" t="n"/>
-      <c r="H73" s="6">
-        <f>IF($G73="","",IF(EDATE(サマリ!$B$2,1)&gt;$G73,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G73,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G73,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I73" s="6" t="n"/>
+      <c r="E73" s="10" t="n"/>
+      <c r="F73" s="6">
+        <f>IF($E73="","",IF(EDATE(サマリ!$B$2,1)&gt;$E73,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E73,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E73,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G73" s="6" t="n"/>
+      <c r="H73" s="6" t="n"/>
+      <c r="I73" s="10" t="n"/>
       <c r="J73" s="6" t="n"/>
       <c r="K73" s="6" t="n"/>
-      <c r="L73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
@@ -4102,17 +3978,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E74" s="6" t="n"/>
-      <c r="F74" s="10" t="n"/>
-      <c r="G74" s="10" t="n"/>
-      <c r="H74" s="6">
-        <f>IF($G74="","",IF(EDATE(サマリ!$B$2,1)&gt;$G74,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G74,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G74,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I74" s="6" t="n"/>
+      <c r="E74" s="10" t="n"/>
+      <c r="F74" s="6">
+        <f>IF($E74="","",IF(EDATE(サマリ!$B$2,1)&gt;$E74,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E74,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E74,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G74" s="6" t="n"/>
+      <c r="H74" s="6" t="n"/>
+      <c r="I74" s="10" t="n"/>
       <c r="J74" s="6" t="n"/>
       <c r="K74" s="6" t="n"/>
-      <c r="L74" s="6" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -4131,17 +4006,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E75" s="6" t="n"/>
-      <c r="F75" s="10" t="n"/>
-      <c r="G75" s="10" t="n"/>
-      <c r="H75" s="6">
-        <f>IF($G75="","",IF(EDATE(サマリ!$B$2,1)&gt;$G75,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G75,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G75,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I75" s="6" t="n"/>
+      <c r="E75" s="10" t="n"/>
+      <c r="F75" s="6">
+        <f>IF($E75="","",IF(EDATE(サマリ!$B$2,1)&gt;$E75,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E75,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E75,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G75" s="6" t="n"/>
+      <c r="H75" s="6" t="n"/>
+      <c r="I75" s="10" t="n"/>
       <c r="J75" s="6" t="n"/>
       <c r="K75" s="6" t="n"/>
-      <c r="L75" s="6" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
@@ -4160,17 +4034,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E76" s="6" t="n"/>
-      <c r="F76" s="10" t="n"/>
-      <c r="G76" s="10" t="n"/>
-      <c r="H76" s="6">
-        <f>IF($G76="","",IF(EDATE(サマリ!$B$2,1)&gt;$G76,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G76,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G76,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I76" s="6" t="n"/>
+      <c r="E76" s="10" t="n"/>
+      <c r="F76" s="6">
+        <f>IF($E76="","",IF(EDATE(サマリ!$B$2,1)&gt;$E76,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E76,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E76,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G76" s="6" t="n"/>
+      <c r="H76" s="6" t="n"/>
+      <c r="I76" s="10" t="n"/>
       <c r="J76" s="6" t="n"/>
       <c r="K76" s="6" t="n"/>
-      <c r="L76" s="6" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
@@ -4189,17 +4062,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E77" s="6" t="n"/>
-      <c r="F77" s="10" t="n"/>
-      <c r="G77" s="10" t="n"/>
-      <c r="H77" s="6">
-        <f>IF($G77="","",IF(EDATE(サマリ!$B$2,1)&gt;$G77,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G77,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G77,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I77" s="6" t="n"/>
+      <c r="E77" s="10" t="n"/>
+      <c r="F77" s="6">
+        <f>IF($E77="","",IF(EDATE(サマリ!$B$2,1)&gt;$E77,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E77,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E77,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G77" s="6" t="n"/>
+      <c r="H77" s="6" t="n"/>
+      <c r="I77" s="10" t="n"/>
       <c r="J77" s="6" t="n"/>
       <c r="K77" s="6" t="n"/>
-      <c r="L77" s="6" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
@@ -4218,17 +4090,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E78" s="6" t="n"/>
-      <c r="F78" s="10" t="n"/>
-      <c r="G78" s="10" t="n"/>
-      <c r="H78" s="6">
-        <f>IF($G78="","",IF(EDATE(サマリ!$B$2,1)&gt;$G78,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G78,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G78,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I78" s="6" t="n"/>
+      <c r="E78" s="10" t="n"/>
+      <c r="F78" s="6">
+        <f>IF($E78="","",IF(EDATE(サマリ!$B$2,1)&gt;$E78,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E78,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E78,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G78" s="6" t="n"/>
+      <c r="H78" s="6" t="n"/>
+      <c r="I78" s="10" t="n"/>
       <c r="J78" s="6" t="n"/>
       <c r="K78" s="6" t="n"/>
-      <c r="L78" s="6" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
@@ -4247,17 +4118,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E79" s="6" t="n"/>
-      <c r="F79" s="10" t="n"/>
-      <c r="G79" s="10" t="n"/>
-      <c r="H79" s="6">
-        <f>IF($G79="","",IF(EDATE(サマリ!$B$2,1)&gt;$G79,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G79,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G79,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I79" s="6" t="n"/>
+      <c r="E79" s="10" t="n"/>
+      <c r="F79" s="6">
+        <f>IF($E79="","",IF(EDATE(サマリ!$B$2,1)&gt;$E79,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E79,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E79,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G79" s="6" t="n"/>
+      <c r="H79" s="6" t="n"/>
+      <c r="I79" s="10" t="n"/>
       <c r="J79" s="6" t="n"/>
       <c r="K79" s="6" t="n"/>
-      <c r="L79" s="6" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
@@ -4276,17 +4146,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E80" s="6" t="n"/>
-      <c r="F80" s="10" t="n"/>
-      <c r="G80" s="10" t="n"/>
-      <c r="H80" s="6">
-        <f>IF($G80="","",IF(EDATE(サマリ!$B$2,1)&gt;$G80,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G80,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G80,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I80" s="6" t="n"/>
+      <c r="E80" s="10" t="n"/>
+      <c r="F80" s="6">
+        <f>IF($E80="","",IF(EDATE(サマリ!$B$2,1)&gt;$E80,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E80,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E80,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G80" s="6" t="n"/>
+      <c r="H80" s="6" t="n"/>
+      <c r="I80" s="10" t="n"/>
       <c r="J80" s="6" t="n"/>
       <c r="K80" s="6" t="n"/>
-      <c r="L80" s="6" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
@@ -4305,17 +4174,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E81" s="6" t="n"/>
-      <c r="F81" s="10" t="n"/>
-      <c r="G81" s="10" t="n"/>
-      <c r="H81" s="6">
-        <f>IF($G81="","",IF(EDATE(サマリ!$B$2,1)&gt;$G81,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G81,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G81,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I81" s="6" t="n"/>
+      <c r="E81" s="10" t="n"/>
+      <c r="F81" s="6">
+        <f>IF($E81="","",IF(EDATE(サマリ!$B$2,1)&gt;$E81,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E81,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E81,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G81" s="6" t="n"/>
+      <c r="H81" s="6" t="n"/>
+      <c r="I81" s="10" t="n"/>
       <c r="J81" s="6" t="n"/>
       <c r="K81" s="6" t="n"/>
-      <c r="L81" s="6" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
@@ -4334,17 +4202,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E82" s="6" t="n"/>
-      <c r="F82" s="10" t="n"/>
-      <c r="G82" s="10" t="n"/>
-      <c r="H82" s="6">
-        <f>IF($G82="","",IF(EDATE(サマリ!$B$2,1)&gt;$G82,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G82,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G82,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I82" s="6" t="n"/>
+      <c r="E82" s="10" t="n"/>
+      <c r="F82" s="6">
+        <f>IF($E82="","",IF(EDATE(サマリ!$B$2,1)&gt;$E82,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E82,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E82,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G82" s="6" t="n"/>
+      <c r="H82" s="6" t="n"/>
+      <c r="I82" s="10" t="n"/>
       <c r="J82" s="6" t="n"/>
       <c r="K82" s="6" t="n"/>
-      <c r="L82" s="6" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
@@ -4363,17 +4230,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E83" s="6" t="n"/>
-      <c r="F83" s="10" t="n"/>
-      <c r="G83" s="10" t="n"/>
-      <c r="H83" s="6">
-        <f>IF($G83="","",IF(EDATE(サマリ!$B$2,1)&gt;$G83,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G83,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G83,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I83" s="6" t="n"/>
+      <c r="E83" s="10" t="n"/>
+      <c r="F83" s="6">
+        <f>IF($E83="","",IF(EDATE(サマリ!$B$2,1)&gt;$E83,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E83,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E83,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G83" s="6" t="n"/>
+      <c r="H83" s="6" t="n"/>
+      <c r="I83" s="10" t="n"/>
       <c r="J83" s="6" t="n"/>
       <c r="K83" s="6" t="n"/>
-      <c r="L83" s="6" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
@@ -4392,17 +4258,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E84" s="6" t="n"/>
-      <c r="F84" s="10" t="n"/>
-      <c r="G84" s="10" t="n"/>
-      <c r="H84" s="6">
-        <f>IF($G84="","",IF(EDATE(サマリ!$B$2,1)&gt;$G84,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G84,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G84,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I84" s="6" t="n"/>
+      <c r="E84" s="10" t="n"/>
+      <c r="F84" s="6">
+        <f>IF($E84="","",IF(EDATE(サマリ!$B$2,1)&gt;$E84,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E84,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E84,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G84" s="6" t="n"/>
+      <c r="H84" s="6" t="n"/>
+      <c r="I84" s="10" t="n"/>
       <c r="J84" s="6" t="n"/>
       <c r="K84" s="6" t="n"/>
-      <c r="L84" s="6" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
@@ -4421,17 +4286,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E85" s="6" t="n"/>
-      <c r="F85" s="10" t="n"/>
-      <c r="G85" s="10" t="n"/>
-      <c r="H85" s="6">
-        <f>IF($G85="","",IF(EDATE(サマリ!$B$2,1)&gt;$G85,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G85,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G85,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I85" s="6" t="n"/>
+      <c r="E85" s="10" t="n"/>
+      <c r="F85" s="6">
+        <f>IF($E85="","",IF(EDATE(サマリ!$B$2,1)&gt;$E85,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E85,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E85,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G85" s="6" t="n"/>
+      <c r="H85" s="6" t="n"/>
+      <c r="I85" s="10" t="n"/>
       <c r="J85" s="6" t="n"/>
       <c r="K85" s="6" t="n"/>
-      <c r="L85" s="6" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr"/>
@@ -4446,17 +4310,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E86" s="6" t="n"/>
-      <c r="F86" s="10" t="n"/>
-      <c r="G86" s="10" t="n"/>
-      <c r="H86" s="6">
-        <f>IF($G86="","",IF(EDATE(サマリ!$B$2,1)&gt;$G86,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G86,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G86,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I86" s="6" t="n"/>
+      <c r="E86" s="10" t="n"/>
+      <c r="F86" s="6">
+        <f>IF($E86="","",IF(EDATE(サマリ!$B$2,1)&gt;$E86,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E86,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E86,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G86" s="6" t="n"/>
+      <c r="H86" s="6" t="n"/>
+      <c r="I86" s="10" t="n"/>
       <c r="J86" s="6" t="n"/>
       <c r="K86" s="6" t="n"/>
-      <c r="L86" s="6" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr"/>
@@ -4471,17 +4334,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E87" s="6" t="n"/>
-      <c r="F87" s="10" t="n"/>
-      <c r="G87" s="10" t="n"/>
-      <c r="H87" s="6">
-        <f>IF($G87="","",IF(EDATE(サマリ!$B$2,1)&gt;$G87,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G87,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G87,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I87" s="6" t="n"/>
+      <c r="E87" s="10" t="n"/>
+      <c r="F87" s="6">
+        <f>IF($E87="","",IF(EDATE(サマリ!$B$2,1)&gt;$E87,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E87,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E87,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G87" s="6" t="n"/>
+      <c r="H87" s="6" t="n"/>
+      <c r="I87" s="10" t="n"/>
       <c r="J87" s="6" t="n"/>
       <c r="K87" s="6" t="n"/>
-      <c r="L87" s="6" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr"/>
@@ -4496,17 +4358,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E88" s="6" t="n"/>
-      <c r="F88" s="10" t="n"/>
-      <c r="G88" s="10" t="n"/>
-      <c r="H88" s="6">
-        <f>IF($G88="","",IF(EDATE(サマリ!$B$2,1)&gt;$G88,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G88,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G88,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I88" s="6" t="n"/>
+      <c r="E88" s="10" t="n"/>
+      <c r="F88" s="6">
+        <f>IF($E88="","",IF(EDATE(サマリ!$B$2,1)&gt;$E88,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E88,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E88,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G88" s="6" t="n"/>
+      <c r="H88" s="6" t="n"/>
+      <c r="I88" s="10" t="n"/>
       <c r="J88" s="6" t="n"/>
       <c r="K88" s="6" t="n"/>
-      <c r="L88" s="6" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr"/>
@@ -4521,17 +4382,16 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E89" s="6" t="n"/>
-      <c r="F89" s="10" t="n"/>
-      <c r="G89" s="10" t="n"/>
-      <c r="H89" s="6">
-        <f>IF($G89="","",IF(EDATE(サマリ!$B$2,1)&gt;$G89,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G89,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G89,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I89" s="6" t="n"/>
+      <c r="E89" s="10" t="n"/>
+      <c r="F89" s="6">
+        <f>IF($E89="","",IF(EDATE(サマリ!$B$2,1)&gt;$E89,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E89,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E89,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G89" s="6" t="n"/>
+      <c r="H89" s="6" t="n"/>
+      <c r="I89" s="10" t="n"/>
       <c r="J89" s="6" t="n"/>
       <c r="K89" s="6" t="n"/>
-      <c r="L89" s="6" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr"/>
@@ -4546,25 +4406,24 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E90" s="6" t="n"/>
-      <c r="F90" s="10" t="n"/>
-      <c r="G90" s="10" t="n"/>
-      <c r="H90" s="6">
-        <f>IF($G90="","",IF(EDATE(サマリ!$B$2,1)&gt;$G90,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$G90,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$G90,"再来月期限",""))))</f>
-        <v/>
-      </c>
-      <c r="I90" s="6" t="n"/>
+      <c r="E90" s="10" t="n"/>
+      <c r="F90" s="6">
+        <f>IF($E90="","",IF(EDATE(サマリ!$B$2,1)&gt;$E90,"期限切れ",IF(EDATE(サマリ!$B$2,2)&gt;$E90,"来月期限",IF(EDATE(サマリ!$B$2,3)&gt;$E90,"再来月期限",""))))</f>
+        <v/>
+      </c>
+      <c r="G90" s="6" t="n"/>
+      <c r="H90" s="6" t="n"/>
+      <c r="I90" s="10" t="n"/>
       <c r="J90" s="6" t="n"/>
       <c r="K90" s="6" t="n"/>
-      <c r="L90" s="6" t="n"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A4:L90">
+  <conditionalFormatting sqref="A4:K90">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$H4="期限切れ"</formula>
+      <formula>$F4="期限切れ"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>$H4="来月期限"</formula>
+      <formula>$F4="来月期限"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C90">
@@ -4572,11 +4431,8 @@
       <formula>ISBLANK($C4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation sqref="J4:J90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=設定!$A$2:$A$11</formula1>
-    </dataValidation>
-    <dataValidation sqref="K4:K90" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1回目完了,ダブルチェック完了"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4590,7 +4446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4598,9 +4454,8 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4649,15 +4504,10 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>入力者</t>
+          <t>チェック</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>チェック</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>備考</t>
         </is>
@@ -4679,7 +4529,6 @@
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
       <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr"/>
@@ -4697,7 +4546,6 @@
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
       <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr"/>
@@ -4715,7 +4563,6 @@
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
       <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr"/>
@@ -4733,7 +4580,6 @@
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr"/>
@@ -4751,7 +4597,6 @@
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr"/>
@@ -4769,7 +4614,6 @@
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr"/>
@@ -4783,7 +4627,6 @@
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr"/>
@@ -4797,7 +4640,6 @@
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr"/>
@@ -4811,7 +4653,6 @@
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr"/>
@@ -4829,7 +4670,6 @@
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr"/>
@@ -4847,7 +4687,6 @@
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr"/>
@@ -4865,7 +4704,6 @@
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr"/>
@@ -4879,7 +4717,6 @@
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr"/>
@@ -4893,7 +4730,6 @@
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D4:E17">
@@ -4901,80 +4737,11 @@
       <formula>AND(ISBLANK($D4),ISBLANK($E4))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation sqref="F4:F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=設定!$A$2:$A$11</formula1>
-    </dataValidation>
-    <dataValidation sqref="G4:G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1回目完了,ダブルチェック完了"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>入力者リスト（自由に書き換えOK・最大10人）</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>入力者A</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>入力者B</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>入力者C</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Convert template sheets to Excel tables for mobile card-view entry
Wrapping each category sheet's data in a ListObject (TBeans/TSubs/
TFilters) lets Excel on iOS/Android offer card view — one item per
form-style card — which is the practical way to make direct entry
usable on phones. Summary tips now tell mobile users to open the file
in the Excel app and switch to card view. Formulas and counters
re-verified after the change.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RgvGiotwKBR4F3r5Tdot14
</commit_message>
<xml_diff>
--- a/excel/棚卸しシート_共同編集版.xlsx
+++ b/excel/棚卸しシート_共同編集版.xlsx
@@ -206,6 +206,62 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TBeans" displayName="TBeans" ref="A3:K41" headerRowCount="1">
+  <autoFilter ref="A3:K41"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="原料コード"/>
+    <tableColumn id="2" name="品名"/>
+    <tableColumn id="3" name="数量"/>
+    <tableColumn id="4" name="単位"/>
+    <tableColumn id="5" name="期限日"/>
+    <tableColumn id="6" name="期限区分(自動)"/>
+    <tableColumn id="7" name="期限量"/>
+    <tableColumn id="8" name="期限切れ量"/>
+    <tableColumn id="9" name="期限切れ日"/>
+    <tableColumn id="10" name="チェック"/>
+    <tableColumn id="11" name="備考"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TSubs" displayName="TSubs" ref="A3:K90" headerRowCount="1">
+  <autoFilter ref="A3:K90"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="原料コード"/>
+    <tableColumn id="2" name="品名"/>
+    <tableColumn id="3" name="数量"/>
+    <tableColumn id="4" name="単位"/>
+    <tableColumn id="5" name="期限日"/>
+    <tableColumn id="6" name="期限区分(自動)"/>
+    <tableColumn id="7" name="期限量"/>
+    <tableColumn id="8" name="期限切れ量"/>
+    <tableColumn id="9" name="期限切れ日"/>
+    <tableColumn id="10" name="チェック"/>
+    <tableColumn id="11" name="備考"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TFilters" displayName="TFilters" ref="A3:G17" headerRowCount="1">
+  <autoFilter ref="A3:G17"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="原料コード"/>
+    <tableColumn id="2" name="品名"/>
+    <tableColumn id="3" name="型番"/>
+    <tableColumn id="4" name="数量(箱)"/>
+    <tableColumn id="5" name="数量(本)"/>
+    <tableColumn id="6" name="チェック"/>
+    <tableColumn id="7" name="備考"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -497,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -720,6 +776,20 @@
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>※ 複数人で同時に開いて編集してOK（自動保存・自動同期）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>★ スマホの人へ: Teamsのプレビューではなく【Excelアプリ】で開き、表の中をタップ →</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   右下に出るカードのアイコンで「カードビュー」にすると1品目=1枚のフォームで入力できます</t>
         </is>
       </c>
     </row>
@@ -1901,6 +1971,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -4437,6 +4510,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -4743,5 +4819,8 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>